<commit_message>
Publish inspected live screenshots and outreach preparation for Bake me mine
</commit_message>
<xml_diff>
--- a/work/office-tracker.xlsx
+++ b/work/office-tracker.xlsx
@@ -602,15 +602,44 @@
           <t>openai/gpt-6-astra</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>60ece4128006ecc83305f28bb660687f636d3df7</t>
+        </is>
+      </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
           <t>https://amalraj020-a11y.github.io/10am-office-work/websites/bake-me-mine-plymouth/</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>["work/screenshots/bake-me-mine-plymouth-desktop.png", "work/screenshots/bake-me-mine-plymouth-mobile.png"]</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hello Bake me mine team,
+I’m Amala from MultiMax. We build affordable websites for local businesses. I came across your Plymouth bakery’s public listings and prepared an independent website concept showing how your custom cakes, cupcakes and cake pops could be presented online. This is an unsolicited demo, not your official website or an endorsement by your business.
+Live preview:
+https://amalraj020-a11y.github.io/10am-office-work/websites/bake-me-mine-plymouth/
+Source code and template/license details:
+https://github.com/amalraj020-a11y/10am-office-work/tree/main/websites/bake-me-mine-plymouth
+I’ve attached two current screenshots: a desktop view and a mobile view. The cake illustration is decorative, not a photograph of your products. Public copies of the screenshots are also here:
+https://amalraj020-a11y.github.io/10am-office-work/work/screenshots/bake-me-mine-plymouth-desktop.png
+https://amalraj020-a11y.github.io/10am-office-work/work/screenshots/bake-me-mine-plymouth-mobile.png
+If the idea is useful, reply and we can discuss your changes and a small, agreed budget. This preview has no online ordering, payment or database system; backend/database features would only be optional later work agreed separately. No payment or commitment is expected for viewing the demo.
+If you’re not interested, just let me know and I won’t follow up.
+Amala
+MultiMax
+</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
           <t>not_attempted</t>
@@ -619,7 +648,7 @@
       <c r="Q2" s="2" t="inlineStr"/>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T18:09:47.008662+00:00</t>
+          <t>2026-10-27T18:11:31.623695+00:00</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Record verified Bake me mine email outreach
</commit_message>
<xml_diff>
--- a/work/office-tracker.xlsx
+++ b/work/office-tracker.xlsx
@@ -642,13 +642,17 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>not_attempted</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>1a17e90d11888e93</t>
+        </is>
+      </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T18:11:31.623695+00:00</t>
+          <t>2026-10-28T12:05:52.281621+00:00</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Add Willow Bakery Kensington independent website concept
</commit_message>
<xml_diff>
--- a/work/office-tracker.xlsx
+++ b/work/office-tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Business work" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Business work'!$A$1:$S$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Business work'!$A$1:$S$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -750,8 +750,81 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>work/the-willow-bakery-kensington/run.json</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>The Willow Bakery &amp; Cafe</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Kensington, Prince Edward Island, Canada</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Bakery and cafe</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>["https://centralcoastalpei.com/members/the-willow-bakery-cafe/", "https://www.tourismpei.com/attractions/the-willow-bakery-cafe", "https://cavendishbeachpei.com/members-operators/the-willow-bakery-cafe/", "https://canadasfoodisland.ca/culinary_trail/the-willow-bakery-cafe/"]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>{"url": "https://centralcoastalpei.com/members/the-willow-bakery-cafe/", "email": "willowhousebakery@gmail.com", "identity_match": "Business name, 13 Commercial Street Kensington address and 902-303-5127 match Tourism PEI and Cavendish Beach listings. Email also appears on Cavendish Beach tourism listing.", "checked_at": "2026-10-29T04:32:28.766653+00:00", "channel": "email", "sender_check": "Configured Gmail OAuth refresh-token check returned valid=true with gmail.send scope in this run.", "confidence": "Public association verified; recipient mailbox delivery unproven."}</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Agency</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>https://themewagon.com/themes/free-bootstrap-5-html-5-business-website-template-agency/</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>MIT; Start Bootstrap and Bootstrap license notices preserved</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>openai/gpt-6-astra</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29T04:35:37.796597+00:00</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S3"/>
+  <autoFilter ref="A1:S4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish verified Willow Bakery screenshots and outreach preparation
</commit_message>
<xml_diff>
--- a/work/office-tracker.xlsx
+++ b/work/office-tracker.xlsx
@@ -801,10 +801,40 @@
           <t>openai/gpt-6-astra</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>b02d5ae4e626ee3a410f392d07723f1d256973b9</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>https://amalraj020-a11y.github.io/10am-office-work/websites/the-willow-bakery-kensington/</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>["work/screenshots/the-willow-bakery-kensington-desktop.png", "work/screenshots/the-willow-bakery-kensington-mobile.png"]</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hello The Willow Bakery &amp; Cafe team,
+I'm Amala from MultiMax. We build affordable websites for local businesses. I came across your Kensington cafe through the PEI tourism listings, which link visitors to your Facebook page, and prepared an independent website concept to show how a dedicated web presence could look.
+The concept brings together your published bakery, coffee and lunch offerings, location and contact details in a mobile-friendly layout. It is clearly marked as an independent preview, not your official website, and uses labelled illustrative photos rather than claiming they show your cafe.
+Live preview:
+https://amalraj020-a11y.github.io/10am-office-work/websites/the-willow-bakery-kensington/
+Source code:
+https://github.com/amalraj020-a11y/10am-office-work/tree/main/websites/the-willow-bakery-kensington
+I've attached two current screenshots, one desktop and one mobile. You can also view them here:
+https://amalraj020-a11y.github.io/10am-office-work/work/screenshots/the-willow-bakery-kensington-desktop.png
+https://amalraj020-a11y.github.io/10am-office-work/work/screenshots/the-willow-bakery-kensington-mobile.png
+If this is useful, reply and we can discuss your preferred photos, wording and a small agreed budget. No purchase or commitment is implied by this preview. Backend or database features could be discussed separately as optional later work; the current concept does not process orders or reservations.
+If you'd prefer not to hear from us, just let me know and I won't follow up.
+Amala
+MultiMax
+</t>
+        </is>
+      </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
           <t>email</t>
@@ -818,7 +848,7 @@
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T04:35:37.796597+00:00</t>
+          <t>2026-10-29T04:38:37.742711+00:00</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Record accepted Willow Bakery email and completed office tracker
</commit_message>
<xml_diff>
--- a/work/office-tracker.xlsx
+++ b/work/office-tracker.xlsx
@@ -842,13 +842,17 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>not_sent</t>
-        </is>
-      </c>
-      <c r="Q4" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>1a185f509ad37707</t>
+        </is>
+      </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T04:38:37.742711+00:00</t>
+          <t>2026-10-29T04:40:21.620518+00:00</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Record Raven's Whisk email acceptance and rebuild office tracker
</commit_message>
<xml_diff>
--- a/work/office-tracker.xlsx
+++ b/work/office-tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Business work" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Business work'!$A$1:$S$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Business work'!$A$1:$S$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S4"/>
+  <dimension ref="A1:S5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -753,70 +753,177 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>work/ravens-whisk-odenton/run.json</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Raven's Whisk Cottage Bakery</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Odenton, Maryland, USA</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Cottage bakery</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>["https://nextdoor.com/pages/ravens-whisk-cottage-bakery/", "https://www.facebook.com/share/18m84ZWt6z/", "https://form.jotform.com/262628079423058"]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>{"url": "https://nextdoor.com/pages/ravens-whisk-cottage-bakery/", "email": "ravenswhiskbakery@gmail.com", "identity_match": "Public business page pairs exact bakery name, Odenton location, phone and email, with business-authored posts and mother/daughter bakery story.", "channel": "email", "checked_at": "2026-10-30T04:32:24.569568+00:00", "sender_check": "Configured Gmail OAuth token exchange returned valid=true and gmail.send scope during this run.", "confidence": "Public association verified; inbox delivery unproven."}</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Stylish Portfolio</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>https://themewagon.com/themes/bootstrap-4-portfolio-template-free-download/</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>MIT; Blackrock Digital / Start Bootstrap and Bootstrap notices preserved</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>openai/gpt-6-astra</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>753fe635cd49eeafbc998d5d63e63a402516861d</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>https://amalraj020-a11y.github.io/10am-office-work/websites/ravens-whisk-odenton/</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>["work/screenshots/ravens-whisk-odenton-desktop.png", "work/screenshots/ravens-whisk-odenton-mobile.png"]</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hello Raven's Whisk team,
+I'm Amala from MultiMax. We build affordable websites for local businesses. I found your Odenton bakery on Nextdoor, where you share your mother-and-daughter story and direct visitors to Facebook. I prepared an independent website concept showing how your bakery could have a dedicated, mobile-friendly introduction.
+The concept brings together your published treats, story and contact details. It is clearly labelled as an independent preview, not your official website. The cookie photograph is labelled illustrative stock photography; your own approved photos could replace it.
+Live preview:
+https://amalraj020-a11y.github.io/10am-office-work/websites/ravens-whisk-odenton/
+Source code:
+https://github.com/amalraj020-a11y/10am-office-work/tree/753fe635cd49eeafbc998d5d63e63a402516861d/websites/ravens-whisk-odenton
+I've attached two current screenshots, one desktop and one mobile. They are also available here:
+https://amalraj020-a11y.github.io/10am-office-work/work/screenshots/ravens-whisk-odenton-desktop.png
+https://amalraj020-a11y.github.io/10am-office-work/work/screenshots/ravens-whisk-odenton-mobile.png
+If you like the direction, reply and we can discuss your preferred wording, photos and a small agreed budget. This preview creates no obligation. It does not process orders or payments; backend or database features would be optional later work, agreed separately.
+If you'd prefer not to hear from us, let me know and I won't follow up.
+Amala
+MultiMax
+</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>1a18b1a825c3d0ee</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30T04:39:10.649791+00:00</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
           <t>work/the-willow-bakery-kensington/run.json</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>The Willow Bakery &amp; Cafe</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Kensington, Prince Edward Island, Canada</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Bakery and cafe</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>["https://centralcoastalpei.com/members/the-willow-bakery-cafe/", "https://www.tourismpei.com/attractions/the-willow-bakery-cafe", "https://cavendishbeachpei.com/members-operators/the-willow-bakery-cafe/", "https://canadasfoodisland.ca/culinary_trail/the-willow-bakery-cafe/"]</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>{"url": "https://centralcoastalpei.com/members/the-willow-bakery-cafe/", "email": "willowhousebakery@gmail.com", "identity_match": "Business name, 13 Commercial Street Kensington address and 902-303-5127 match Tourism PEI and Cavendish Beach listings. Email also appears on Cavendish Beach tourism listing.", "checked_at": "2026-10-29T04:32:28.766653+00:00", "channel": "email", "sender_check": "Configured Gmail OAuth refresh-token check returned valid=true with gmail.send scope in this run.", "confidence": "Public association verified; recipient mailbox delivery unproven."}</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>https://themewagon.com/themes/free-bootstrap-5-html-5-business-website-template-agency/</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>MIT; Start Bootstrap and Bootstrap license notices preserved</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>openai/gpt-6-astra</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>b02d5ae4e626ee3a410f392d07723f1d256973b9</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>https://amalraj020-a11y.github.io/10am-office-work/websites/the-willow-bakery-kensington/</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>["work/screenshots/the-willow-bakery-kensington-desktop.png", "work/screenshots/the-willow-bakery-kensington-mobile.png"]</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Hello The Willow Bakery &amp; Cafe team,
 I'm Amala from MultiMax. We build affordable websites for local businesses. I came across your Kensington cafe through the PEI tourism listings, which link visitors to your Facebook page, and prepared an independent website concept to show how a dedicated web presence could look.
@@ -835,30 +942,30 @@
 </t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>accepted</t>
         </is>
       </c>
-      <c r="Q4" s="2" t="inlineStr">
+      <c r="Q5" s="2" t="inlineStr">
         <is>
           <t>1a185f509ad37707</t>
         </is>
       </c>
-      <c r="R4" s="2" t="inlineStr">
+      <c r="R5" s="2" t="inlineStr">
         <is>
           <t>2026-10-29T04:40:21.620518+00:00</t>
         </is>
       </c>
-      <c r="S4" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S4"/>
+  <autoFilter ref="A1:S5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish verified live screenshots and QA for Sierra's bakery
</commit_message>
<xml_diff>
--- a/work/office-tracker.xlsx
+++ b/work/office-tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Business work" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Business work'!$A$1:$S$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Business work'!$A$1:$S$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S5"/>
+  <dimension ref="A1:S6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -860,70 +860,173 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>work/sierras-baked-goods-nicholasville/run.json</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Sierra's Baked Goods</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Nicholasville, Kentucky, United States</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Cottage bakery</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>["https://nextdoor.com/pages/sierras-baked-goods/", "https://www.facebook.com/people/Sierras-Baked-Goods/61593717573727/", "https://happeningnext.com/event/sierras-marksbury-farm-eid3a0e6jfhbo"]</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>https://nextdoor.com/pages/sierras-baked-goods/</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>New Age</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>https://themewagon.com/themes/free-responsive-one-page-app-landing-bootstrap-template-download-2017/</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>MIT; Start Bootstrap New Age v6.0.1; Bootstrap 5.0.1 MIT</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>openai/gpt-6-astra</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>5e182eab7a7d1a660a970a59adfb0ae554cbb07f</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>https://amalraj020-a11y.github.io/10am-office-work/websites/sierras-baked-goods-nicholasville/</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>["work/screenshots/sierras-baked-goods-nicholasville-desktop.png", "work/screenshots/sierras-baked-goods-nicholasville-mobile.png"]</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hello Sierra's Baked Goods team,
+I'm Amala from MultiMax. We build affordable websites for local businesses. I came across your Nicholasville bakery's public Nextdoor listing and Facebook profile, and prepared an independent website concept for your mini loaves, gourmet brownies, cake pops, and custom party orders.
+I didn't find a dedicated official website in the public sources I checked. This is an unsolicited concept for your review, not your official website or an endorsement by you. The bakery illustration is decorative, not a photograph of your products. The preview does not take orders or payments.
+Live preview:
+https://amalraj020-a11y.github.io/10am-office-work/websites/sierras-baked-goods-nicholasville/
+Source code and license:
+https://github.com/amalraj020-a11y/10am-office-work/tree/5e182eab7a7d1a660a970a59adfb0ae554cbb07f/websites/sierras-baked-goods-nicholasville
+I've attached two current screenshots of the live preview, one desktop and one mobile. You can also view them here:
+https://amalraj020-a11y.github.io/10am-office-work/work/screenshots/sierras-baked-goods-nicholasville-desktop.png
+https://amalraj020-a11y.github.io/10am-office-work/work/screenshots/sierras-baked-goods-nicholasville-mobile.png
+If the direction appeals to you, reply and we can discuss the changes you want and a small agreed budget. There is no obligation. Backend or database features would be optional later work, separately agreed.
+If this isn't relevant, let me know and I won't contact you again.
+Amala
+MultiMax
+</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31T04:38:02.937428+00:00</t>
+        </is>
+      </c>
+      <c r="S5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
           <t>work/the-willow-bakery-kensington/run.json</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>The Willow Bakery &amp; Cafe</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Kensington, Prince Edward Island, Canada</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Bakery and cafe</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>["https://centralcoastalpei.com/members/the-willow-bakery-cafe/", "https://www.tourismpei.com/attractions/the-willow-bakery-cafe", "https://cavendishbeachpei.com/members-operators/the-willow-bakery-cafe/", "https://canadasfoodisland.ca/culinary_trail/the-willow-bakery-cafe/"]</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>{"url": "https://centralcoastalpei.com/members/the-willow-bakery-cafe/", "email": "willowhousebakery@gmail.com", "identity_match": "Business name, 13 Commercial Street Kensington address and 902-303-5127 match Tourism PEI and Cavendish Beach listings. Email also appears on Cavendish Beach tourism listing.", "checked_at": "2026-10-29T04:32:28.766653+00:00", "channel": "email", "sender_check": "Configured Gmail OAuth refresh-token check returned valid=true with gmail.send scope in this run.", "confidence": "Public association verified; recipient mailbox delivery unproven."}</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Agency</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>https://themewagon.com/themes/free-bootstrap-5-html-5-business-website-template-agency/</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>MIT; Start Bootstrap and Bootstrap license notices preserved</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>openai/gpt-6-astra</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>b02d5ae4e626ee3a410f392d07723f1d256973b9</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>https://amalraj020-a11y.github.io/10am-office-work/websites/the-willow-bakery-kensington/</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>["work/screenshots/the-willow-bakery-kensington-desktop.png", "work/screenshots/the-willow-bakery-kensington-mobile.png"]</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Hello The Willow Bakery &amp; Cafe team,
 I'm Amala from MultiMax. We build affordable websites for local businesses. I came across your Kensington cafe through the PEI tourism listings, which link visitors to your Facebook page, and prepared an independent website concept to show how a dedicated web presence could look.
@@ -942,30 +1045,30 @@
 </t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>accepted</t>
         </is>
       </c>
-      <c r="Q5" s="2" t="inlineStr">
+      <c r="Q6" s="2" t="inlineStr">
         <is>
           <t>1a185f509ad37707</t>
         </is>
       </c>
-      <c r="R5" s="2" t="inlineStr">
+      <c r="R6" s="2" t="inlineStr">
         <is>
           <t>2026-10-29T04:40:21.620518+00:00</t>
         </is>
       </c>
-      <c r="S5" s="2" t="inlineStr"/>
+      <c r="S6" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S5"/>
+  <autoFilter ref="A1:S6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record accepted Sierra's bakery outreach and final tracker
</commit_message>
<xml_diff>
--- a/work/office-tracker.xlsx
+++ b/work/office-tracker.xlsx
@@ -949,13 +949,17 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>not_sent</t>
-        </is>
-      </c>
-      <c r="Q5" s="2" t="inlineStr"/>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>1a1904109d88fb6e</t>
+        </is>
+      </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31T04:38:02.937428+00:00</t>
+          <t>2026-10-31T04:39:24.636631+00:00</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr"/>

</xml_diff>